<commit_message>
Feat: add widgets for data_loader
</commit_message>
<xml_diff>
--- a/data/data_cat.xlsx
+++ b/data/data_cat.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -283,13 +283,13 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="str">
         <f t="shared" ref="A2:A33" ca="1" si="0">IF(RAND()&gt;=0.5,"yes","no")</f>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
@@ -301,7 +301,7 @@
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
@@ -313,13 +313,13 @@
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
@@ -331,19 +331,19 @@
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
@@ -355,7 +355,7 @@
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
@@ -367,13 +367,13 @@
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
@@ -391,19 +391,19 @@
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
@@ -415,7 +415,7 @@
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
@@ -427,7 +427,7 @@
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
@@ -451,13 +451,13 @@
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
@@ -475,7 +475,7 @@
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="str">
         <f t="shared" ref="A34:A65" ca="1" si="1">IF(RAND()&gt;=0.5,"yes","no")</f>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
@@ -487,7 +487,7 @@
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
@@ -505,13 +505,13 @@
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
@@ -535,13 +535,13 @@
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
@@ -553,7 +553,7 @@
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
@@ -565,7 +565,7 @@
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
@@ -577,13 +577,13 @@
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
@@ -595,31 +595,31 @@
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
@@ -637,25 +637,25 @@
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
@@ -679,7 +679,7 @@
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
@@ -697,13 +697,13 @@
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
@@ -727,7 +727,7 @@
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
@@ -739,25 +739,25 @@
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
@@ -775,13 +775,13 @@
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
@@ -793,7 +793,7 @@
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
@@ -805,13 +805,13 @@
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
@@ -823,13 +823,13 @@
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
@@ -841,7 +841,7 @@
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.35">
@@ -853,13 +853,13 @@
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" t="str">
         <f t="shared" ref="A98:A129" ca="1" si="3">IF(RAND()&gt;=0.5,"yes","no")</f>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.35">
@@ -883,7 +883,7 @@
     <row r="102" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.35">
@@ -895,13 +895,13 @@
     <row r="104" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.35">
@@ -925,7 +925,7 @@
     <row r="109" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.35">
@@ -943,7 +943,7 @@
     <row r="112" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.35">
@@ -967,7 +967,7 @@
     <row r="116" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.35">
@@ -985,7 +985,7 @@
     <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.35">
@@ -1009,13 +1009,13 @@
     <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.35">
@@ -1033,7 +1033,7 @@
     <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.35">
@@ -1063,13 +1063,13 @@
     <row r="132" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A132" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.35">
@@ -1081,13 +1081,13 @@
     <row r="135" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A136" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.35">
@@ -1099,7 +1099,7 @@
     <row r="138" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.35">
@@ -1117,13 +1117,13 @@
     <row r="141" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A141" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.35">
@@ -1141,7 +1141,7 @@
     <row r="145" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.35">
@@ -1153,13 +1153,13 @@
     <row r="147" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.35">
@@ -1201,7 +1201,7 @@
     <row r="155" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.35">
@@ -1225,13 +1225,13 @@
     <row r="159" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.35">
@@ -1243,7 +1243,7 @@
     <row r="162" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.35">
@@ -1261,7 +1261,7 @@
     <row r="165" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.35">
@@ -1273,7 +1273,7 @@
     <row r="167" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.35">
@@ -1291,13 +1291,13 @@
     <row r="170" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A170" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.35">
@@ -1309,7 +1309,7 @@
     <row r="173" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.35">
@@ -1321,13 +1321,13 @@
     <row r="175" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.35">
@@ -1339,7 +1339,7 @@
     <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.35">
@@ -1375,7 +1375,7 @@
     <row r="184" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.35">
@@ -1387,7 +1387,7 @@
     <row r="186" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.35">
@@ -1399,13 +1399,13 @@
     <row r="188" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.35">
@@ -1417,7 +1417,7 @@
     <row r="191" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.35">
@@ -1429,13 +1429,13 @@
     <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" t="str">
         <f t="shared" ref="A194:A200" ca="1" si="5">IF(RAND()&gt;=0.5,"yes","no")</f>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.35">
@@ -1453,13 +1453,13 @@
     <row r="197" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.35">
@@ -1497,19 +1497,19 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="str">
         <f ca="1">IF(RAND()&lt;1/3,"yes",IF(RAND()&gt;1/2,"no", "idk"))</f>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A66" ca="1" si="0">IF(RAND()&lt;0.33,"yes",IF(RAND()&gt;=0.5,"no", "idk"))</f>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
@@ -1545,49 +1545,49 @@
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
@@ -1599,37 +1599,37 @@
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
@@ -1647,19 +1647,19 @@
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
@@ -1671,19 +1671,19 @@
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
@@ -1713,19 +1713,19 @@
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
@@ -1743,13 +1743,13 @@
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
@@ -1767,13 +1767,13 @@
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
@@ -1785,13 +1785,13 @@
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
@@ -1803,19 +1803,19 @@
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
@@ -1827,13 +1827,13 @@
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
@@ -1845,7 +1845,7 @@
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
@@ -1863,19 +1863,19 @@
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.35">
@@ -1887,43 +1887,43 @@
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="str">
         <f t="shared" ref="A67:A130" ca="1" si="1">IF(RAND()&lt;0.33,"yes",IF(RAND()&gt;=0.5,"no", "idk"))</f>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
@@ -1935,79 +1935,79 @@
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
@@ -2019,13 +2019,13 @@
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
@@ -2037,31 +2037,31 @@
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
@@ -2073,13 +2073,13 @@
     <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.35">
@@ -2091,19 +2091,19 @@
     <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.35">
@@ -2115,13 +2115,13 @@
     <row r="105" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A105" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.35">
@@ -2139,25 +2139,25 @@
     <row r="109" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.35">
@@ -2175,7 +2175,7 @@
     <row r="115" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.35">
@@ -2199,43 +2199,43 @@
     <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.35">
@@ -2247,13 +2247,13 @@
     <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.35">
@@ -2265,25 +2265,25 @@
     <row r="130" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A131" t="str">
         <f t="shared" ref="A131:A194" ca="1" si="2">IF(RAND()&lt;0.33,"yes",IF(RAND()&gt;=0.5,"no", "idk"))</f>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A132" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.35">
@@ -2313,19 +2313,19 @@
     <row r="138" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.35">
@@ -2337,19 +2337,19 @@
     <row r="142" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A142" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.35">
@@ -2361,19 +2361,19 @@
     <row r="146" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A147" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A148" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.35">
@@ -2385,25 +2385,25 @@
     <row r="150" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A153" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.35">
@@ -2415,49 +2415,49 @@
     <row r="155" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A158" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A160" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A161" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A162" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.35">
@@ -2475,7 +2475,7 @@
     <row r="165" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.35">
@@ -2487,55 +2487,55 @@
     <row r="167" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A169" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A170" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A171" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A173" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.35">
@@ -2547,43 +2547,43 @@
     <row r="177" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A181" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.35">
@@ -2601,7 +2601,7 @@
     <row r="186" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A186" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.35">
@@ -2613,19 +2613,19 @@
     <row r="188" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A188" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.35">
@@ -2637,25 +2637,25 @@
     <row r="192" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A195" t="str">
         <f t="shared" ref="A195:A200" ca="1" si="3">IF(RAND()&lt;0.33,"yes",IF(RAND()&gt;=0.5,"no", "idk"))</f>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.35">
@@ -2667,13 +2667,13 @@
     <row r="197" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A197" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.35">
@@ -2685,7 +2685,7 @@
     <row r="200" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
   </sheetData>
@@ -2711,7 +2711,7 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="str">
         <f ca="1">IF(RAND()&gt;=0.3,"yes","no")</f>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
@@ -2723,7 +2723,7 @@
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
@@ -2753,7 +2753,7 @@
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
@@ -2771,7 +2771,7 @@
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
@@ -2795,7 +2795,7 @@
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
@@ -2813,13 +2813,13 @@
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
@@ -2855,13 +2855,13 @@
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
@@ -2873,7 +2873,7 @@
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
@@ -2921,7 +2921,7 @@
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
@@ -2933,7 +2933,7 @@
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
@@ -2945,7 +2945,7 @@
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
@@ -2969,13 +2969,13 @@
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
@@ -2987,13 +2987,13 @@
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
@@ -3005,13 +3005,13 @@
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
@@ -3023,25 +3023,25 @@
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
@@ -3053,13 +3053,13 @@
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
@@ -3101,7 +3101,7 @@
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="str">
         <f t="shared" ref="A67:A130" ca="1" si="1">IF(RAND()&gt;=0.3,"yes","no")</f>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
@@ -3113,13 +3113,13 @@
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
@@ -3131,13 +3131,13 @@
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
@@ -3161,19 +3161,19 @@
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
@@ -3215,25 +3215,25 @@
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
@@ -3245,13 +3245,13 @@
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
@@ -3281,7 +3281,7 @@
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.35">
@@ -3299,13 +3299,13 @@
     <row r="100" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.35">
@@ -3317,7 +3317,7 @@
     <row r="103" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A103" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.35">
@@ -3335,13 +3335,13 @@
     <row r="106" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A106" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A107" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.35">
@@ -3365,13 +3365,13 @@
     <row r="111" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A112" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.35">
@@ -3401,19 +3401,19 @@
     <row r="117" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.35">
@@ -3425,7 +3425,7 @@
     <row r="121" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.35">
@@ -3437,31 +3437,31 @@
     <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A126" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.35">
@@ -3479,7 +3479,7 @@
     <row r="130" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A130" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.35">
@@ -3491,7 +3491,7 @@
     <row r="132" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A132" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.35">
@@ -3509,7 +3509,7 @@
     <row r="135" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.35">
@@ -3521,7 +3521,7 @@
     <row r="137" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.35">
@@ -3563,13 +3563,13 @@
     <row r="144" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.35">
@@ -3599,13 +3599,13 @@
     <row r="150" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.35">
@@ -3629,7 +3629,7 @@
     <row r="155" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A155" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.35">
@@ -3641,7 +3641,7 @@
     <row r="157" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A157" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.35">
@@ -3677,7 +3677,7 @@
     <row r="163" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.35">
@@ -3689,19 +3689,19 @@
     <row r="165" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A165" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A167" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.35">
@@ -3713,7 +3713,7 @@
     <row r="169" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A169" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.35">
@@ -3731,7 +3731,7 @@
     <row r="172" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.35">
@@ -3743,7 +3743,7 @@
     <row r="174" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.35">
@@ -3761,13 +3761,13 @@
     <row r="177" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.35">
@@ -3779,7 +3779,7 @@
     <row r="180" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.35">
@@ -3791,13 +3791,13 @@
     <row r="182" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.35">
@@ -3821,7 +3821,7 @@
     <row r="187" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.35">
@@ -3845,13 +3845,13 @@
     <row r="191" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.35">
@@ -3863,7 +3863,7 @@
     <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.35">
@@ -3887,13 +3887,13 @@
     <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A199" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.35">
@@ -3931,25 +3931,25 @@
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A66" ca="1" si="0">IF(RAND()&lt;1/2,"yes",IF(RAND()&gt;1/2,"no", "idk"))</f>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
@@ -3961,7 +3961,7 @@
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
@@ -3973,61 +3973,61 @@
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
@@ -4045,13 +4045,13 @@
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
@@ -4075,7 +4075,7 @@
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
@@ -4087,7 +4087,7 @@
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
@@ -4099,7 +4099,7 @@
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
@@ -4111,7 +4111,7 @@
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
@@ -4123,13 +4123,13 @@
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
@@ -4141,7 +4141,7 @@
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
@@ -4153,7 +4153,7 @@
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
@@ -4171,13 +4171,13 @@
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
@@ -4195,13 +4195,13 @@
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
@@ -4213,25 +4213,25 @@
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
@@ -4249,7 +4249,7 @@
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
@@ -4261,19 +4261,19 @@
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
@@ -4285,43 +4285,43 @@
     <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="str">
         <f t="shared" ref="A67:A130" ca="1" si="1">IF(RAND()&lt;1/2,"yes",IF(RAND()&gt;1/2,"no", "idk"))</f>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
@@ -4339,7 +4339,7 @@
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
@@ -4351,13 +4351,13 @@
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
@@ -4369,7 +4369,7 @@
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
@@ -4387,25 +4387,25 @@
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
@@ -4417,19 +4417,19 @@
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
@@ -4441,13 +4441,13 @@
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
@@ -4465,13 +4465,13 @@
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
@@ -4483,7 +4483,7 @@
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.35">
@@ -4501,31 +4501,31 @@
     <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A99" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A100" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A102" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.35">
@@ -4537,7 +4537,7 @@
     <row r="104" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A104" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.35">
@@ -4567,19 +4567,19 @@
     <row r="109" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A109" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A110" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A111" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.35">
@@ -4597,73 +4597,73 @@
     <row r="114" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A114" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A115" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A116" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A117" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A118" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A120" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A121" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A122" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A125" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.35">
@@ -4675,13 +4675,13 @@
     <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A128" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.35">
@@ -4699,7 +4699,7 @@
     <row r="131" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A131" t="str">
         <f t="shared" ref="A131:A194" ca="1" si="2">IF(RAND()&lt;1/2,"yes",IF(RAND()&gt;1/2,"no", "idk"))</f>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.35">
@@ -4711,7 +4711,7 @@
     <row r="133" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A133" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.35">
@@ -4723,7 +4723,7 @@
     <row r="135" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A135" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.35">
@@ -4735,25 +4735,25 @@
     <row r="137" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A137" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A138" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A139" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A140" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.35">
@@ -4771,25 +4771,25 @@
     <row r="143" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A143" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A144" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A145" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A146" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.35">
@@ -4813,19 +4813,19 @@
     <row r="150" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A150" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A151" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A152" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.35">
@@ -4849,7 +4849,7 @@
     <row r="156" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A156" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.35">
@@ -4867,7 +4867,7 @@
     <row r="159" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A159" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.35">
@@ -4891,7 +4891,7 @@
     <row r="163" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A163" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.35">
@@ -4909,7 +4909,7 @@
     <row r="166" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A166" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.35">
@@ -4921,19 +4921,19 @@
     <row r="168" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A168" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A169" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A170" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.35">
@@ -4945,7 +4945,7 @@
     <row r="172" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A172" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.35">
@@ -4957,43 +4957,43 @@
     <row r="174" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A174" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A175" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A176" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A177" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A179" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A180" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.35">
@@ -5005,19 +5005,19 @@
     <row r="182" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A182" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A184" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.35">
@@ -5035,7 +5035,7 @@
     <row r="187" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A187" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.35">
@@ -5047,49 +5047,49 @@
     <row r="189" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A189" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A190" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>yes</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A191" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>no</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A192" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>no</v>
+        <v>idk</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A195" t="str">
         <f t="shared" ref="A195:A200" ca="1" si="3">IF(RAND()&lt;1/2,"yes",IF(RAND()&gt;1/2,"no", "idk"))</f>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A196" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>idk</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.35">
@@ -5113,7 +5113,7 @@
     <row r="200" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A200" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
   </sheetData>

</xml_diff>